<commit_message>
docs: refresh all-pages screenshot sweep post P0-fix deploy (83/83 ok) + fix summary double-write in shoot script
</commit_message>
<xml_diff>
--- a/docs/user-guide/screenshots/all-pages/export-excel.xlsx
+++ b/docs/user-guide/screenshots/all-pages/export-excel.xlsx
@@ -477,7 +477,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ingrediente 7ec03f12</t>
+          <t>Ingrediente ac7a9c2a</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Receta 2f6bbb5d</t>
+          <t>Receta 3117c905</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -682,7 +682,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Receta 2f6bbb5d</t>
+          <t>Receta 3117c905</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Ingrediente 7ec03f12</t>
+          <t>Ingrediente ac7a9c2a</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -797,7 +797,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Producto 5bf8a725</t>
+          <t>Producto 7e132b24</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Receta 2f6bbb5d</t>
+          <t>Receta 3117c905</t>
         </is>
       </c>
     </row>
@@ -999,14 +999,14 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46287.84018083566</v>
+        <v>46287.87390256486</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Producto 5bf8a725</t>
+          <t>Producto 7e132b24</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1023,14 +1023,14 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46288.17351416899</v>
+        <v>46288.2072358982</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Producto 5bf8a725</t>
+          <t>Producto 7e132b24</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1047,14 +1047,14 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46288.50684750233</v>
+        <v>46288.54056923153</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Producto 5bf8a725</t>
+          <t>Producto 7e132b24</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1071,14 +1071,14 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46288.84018083566</v>
+        <v>46288.87390256486</v>
       </c>
       <c r="C5" t="n">
         <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Producto 5bf8a725</t>
+          <t>Producto 7e132b24</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1095,14 +1095,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46289.17351416899</v>
+        <v>46289.2072358982</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Producto 5bf8a725</t>
+          <t>Producto 7e132b24</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1119,14 +1119,14 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46289.50684750233</v>
+        <v>46289.54056923153</v>
       </c>
       <c r="C7" t="n">
         <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Producto 5bf8a725</t>
+          <t>Producto 7e132b24</t>
         </is>
       </c>
       <c r="E7" t="n">

</xml_diff>

<commit_message>
UI redesign: app shell (sidebar+topbar), Inicio v3 (HOY+Acciones+Alertas+Plan), /analisis analytics page, Inventario KPI strip+filters+health bars
- base.html rewritten: persistent sidebar >=1024px (Operacion/Catalogo/Compras/Finanzas/Sistema), topbar clock+search+ Nuevo dropdown, login keeps old chrome
- app-shell.css new
- inicio.html v3: greeting hero, HOY KPI band vs same weekday, Acciones del dia checklist, capped Alertas with severity pills, Plan de manana, Analisis teaser
- analisis.py + analisis.html: analytics destination (stars/dogs, rising/churning, price fluctuation, erosion, turnover, dow, complexity)
- inventario: KPI strip (total/critico/valor/sin costo), filter toolbar (q/categoria/estado), stock health micro-bars
- dashboard.py: tz-safe same-weekday comparison, acciones queries, ticket/ops KPIs
- browser pages.py: sidebar selectors replace hamburger
- 20 stale tests updated to new nav/analytics contracts; suite21 2315/0, browser 9/9
</commit_message>
<xml_diff>
--- a/docs/user-guide/screenshots/all-pages/export-excel.xlsx
+++ b/docs/user-guide/screenshots/all-pages/export-excel.xlsx
@@ -477,7 +477,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ingrediente ac7a9c2a</t>
+          <t>Ingrediente f910ed0e</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Receta 3117c905</t>
+          <t>Receta dd5d03e8</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -682,7 +682,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Receta 3117c905</t>
+          <t>Receta dd5d03e8</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Ingrediente ac7a9c2a</t>
+          <t>Ingrediente f910ed0e</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -797,7 +797,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Producto 7e132b24</t>
+          <t>Producto 4d6e202a</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Receta 3117c905</t>
+          <t>Receta dd5d03e8</t>
         </is>
       </c>
     </row>
@@ -999,14 +999,14 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46287.87390256486</v>
+        <v>46287.9705130111</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Producto 7e132b24</t>
+          <t>Producto 4d6e202a</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1023,14 +1023,14 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46288.2072358982</v>
+        <v>46288.30384634443</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Producto 7e132b24</t>
+          <t>Producto 4d6e202a</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1047,14 +1047,14 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46288.54056923153</v>
+        <v>46288.63717967777</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Producto 7e132b24</t>
+          <t>Producto 4d6e202a</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1071,14 +1071,14 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46288.87390256486</v>
+        <v>46288.9705130111</v>
       </c>
       <c r="C5" t="n">
         <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Producto 7e132b24</t>
+          <t>Producto 4d6e202a</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1095,14 +1095,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46289.2072358982</v>
+        <v>46289.30384634443</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Producto 7e132b24</t>
+          <t>Producto 4d6e202a</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1119,14 +1119,14 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46289.54056923153</v>
+        <v>46289.63717967777</v>
       </c>
       <c r="C7" t="n">
         <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Producto 7e132b24</t>
+          <t>Producto 4d6e202a</t>
         </is>
       </c>
       <c r="E7" t="n">

</xml_diff>

<commit_message>
Shell QA fixes: search pill inline ?/Cmd+K (nested button bug), Spanish now_str, (c) footer, humanize hash product names in Plan de manana
</commit_message>
<xml_diff>
--- a/docs/user-guide/screenshots/all-pages/export-excel.xlsx
+++ b/docs/user-guide/screenshots/all-pages/export-excel.xlsx
@@ -477,7 +477,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ingrediente f910ed0e</t>
+          <t>Ingrediente 038f06df</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Receta dd5d03e8</t>
+          <t>Receta 5ea80280</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -682,7 +682,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Receta dd5d03e8</t>
+          <t>Receta 5ea80280</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Ingrediente f910ed0e</t>
+          <t>Ingrediente 038f06df</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -797,7 +797,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Producto 4d6e202a</t>
+          <t>Producto d02a8eb4</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Receta dd5d03e8</t>
+          <t>Receta 5ea80280</t>
         </is>
       </c>
     </row>
@@ -999,14 +999,14 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46287.9705130111</v>
+        <v>46288.22342887763</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Producto 4d6e202a</t>
+          <t>Producto d02a8eb4</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1023,14 +1023,14 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46288.30384634443</v>
+        <v>46288.55676221096</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Producto 4d6e202a</t>
+          <t>Producto d02a8eb4</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1047,14 +1047,14 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46288.63717967777</v>
+        <v>46288.8900955443</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Producto 4d6e202a</t>
+          <t>Producto d02a8eb4</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1071,14 +1071,14 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46288.9705130111</v>
+        <v>46289.22342887763</v>
       </c>
       <c r="C5" t="n">
         <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Producto 4d6e202a</t>
+          <t>Producto d02a8eb4</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1095,14 +1095,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46289.30384634443</v>
+        <v>46289.55676221096</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Producto 4d6e202a</t>
+          <t>Producto d02a8eb4</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1119,14 +1119,14 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46289.63717967777</v>
+        <v>46289.8900955443</v>
       </c>
       <c r="C7" t="n">
         <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Producto 4d6e202a</t>
+          <t>Producto d02a8eb4</t>
         </is>
       </c>
       <c r="E7" t="n">

</xml_diff>

<commit_message>
Audit round 2 fixes: Gs. currency unification (9 templates had wrong PYG glyph), honest margen/food-cost (sin escandallo instead of 100%/0%), pedidos tabs instead of stacked sections, login professional microcopy, receta-detalle dedup table
</commit_message>
<xml_diff>
--- a/docs/user-guide/screenshots/all-pages/export-excel.xlsx
+++ b/docs/user-guide/screenshots/all-pages/export-excel.xlsx
@@ -477,7 +477,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ingrediente 038f06df</t>
+          <t>Ingrediente cb3902ac</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Receta 5ea80280</t>
+          <t>Receta e2d0d7f1</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -682,7 +682,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Receta 5ea80280</t>
+          <t>Receta e2d0d7f1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Ingrediente 038f06df</t>
+          <t>Ingrediente cb3902ac</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -797,7 +797,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Producto d02a8eb4</t>
+          <t>Producto 82181abe</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Receta 5ea80280</t>
+          <t>Receta e2d0d7f1</t>
         </is>
       </c>
     </row>
@@ -999,14 +999,14 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46288.22342887763</v>
+        <v>46288.26570425607</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Producto d02a8eb4</t>
+          <t>Producto 82181abe</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1023,14 +1023,14 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46288.55676221096</v>
+        <v>46288.59903758941</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Producto d02a8eb4</t>
+          <t>Producto 82181abe</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1047,14 +1047,14 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46288.8900955443</v>
+        <v>46288.93237092275</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Producto d02a8eb4</t>
+          <t>Producto 82181abe</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1071,14 +1071,14 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46289.22342887763</v>
+        <v>46289.26570425607</v>
       </c>
       <c r="C5" t="n">
         <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Producto d02a8eb4</t>
+          <t>Producto 82181abe</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1095,14 +1095,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46289.55676221096</v>
+        <v>46289.59903758941</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Producto d02a8eb4</t>
+          <t>Producto 82181abe</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1119,14 +1119,14 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46289.8900955443</v>
+        <v>46289.93237092275</v>
       </c>
       <c r="C7" t="n">
         <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Producto d02a8eb4</t>
+          <t>Producto 82181abe</t>
         </is>
       </c>
       <c r="E7" t="n">

</xml_diff>

<commit_message>
Inicio dedup round 3: single stock-low surface (Alertas pill row), compliance banner folded into Alertas, Avisos section slimmed, main content max-width 1440px
</commit_message>
<xml_diff>
--- a/docs/user-guide/screenshots/all-pages/export-excel.xlsx
+++ b/docs/user-guide/screenshots/all-pages/export-excel.xlsx
@@ -477,7 +477,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ingrediente cb3902ac</t>
+          <t>Ingrediente 59446791</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Receta e2d0d7f1</t>
+          <t>Receta 7dab5b64</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -682,7 +682,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Receta e2d0d7f1</t>
+          <t>Receta 7dab5b64</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Ingrediente cb3902ac</t>
+          <t>Ingrediente 59446791</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -797,7 +797,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Producto 82181abe</t>
+          <t>Producto 27078bf6</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Receta e2d0d7f1</t>
+          <t>Receta 7dab5b64</t>
         </is>
       </c>
     </row>
@@ -999,14 +999,14 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46288.26570425607</v>
+        <v>46288.29523119341</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Producto 82181abe</t>
+          <t>Producto 27078bf6</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1023,14 +1023,14 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46288.59903758941</v>
+        <v>46288.62856452673</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Producto 82181abe</t>
+          <t>Producto 27078bf6</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1047,14 +1047,14 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46288.93237092275</v>
+        <v>46288.96189786007</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Producto 82181abe</t>
+          <t>Producto 27078bf6</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1071,14 +1071,14 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46289.26570425607</v>
+        <v>46289.29523119341</v>
       </c>
       <c r="C5" t="n">
         <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Producto 82181abe</t>
+          <t>Producto 27078bf6</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1095,14 +1095,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46289.59903758941</v>
+        <v>46289.62856452673</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Producto 82181abe</t>
+          <t>Producto 27078bf6</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1119,14 +1119,14 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46289.93237092275</v>
+        <v>46289.96189786007</v>
       </c>
       <c r="C7" t="n">
         <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Producto 82181abe</t>
+          <t>Producto 27078bf6</t>
         </is>
       </c>
       <c r="E7" t="n">

</xml_diff>

<commit_message>
Phase 0 setup: nav SSOT (NAV_GROUPS/CRUMBS/STATUS_MAP drive sidebar+crumbs+menu), fmt.* formatters (F1-F7), atoms.html (16 macros A1-A16), app-components css/js (drawer/pills/strip/stepper/timer/heatmap), base.html renders from SSOT, 28 acceptance tests (suite 2343/0)
</commit_message>
<xml_diff>
--- a/docs/user-guide/screenshots/all-pages/export-excel.xlsx
+++ b/docs/user-guide/screenshots/all-pages/export-excel.xlsx
@@ -477,7 +477,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ingrediente 59446791</t>
+          <t>Ingrediente 9551f65b</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Receta 7dab5b64</t>
+          <t>Receta 0e8c932f</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -682,7 +682,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Receta 7dab5b64</t>
+          <t>Receta 0e8c932f</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Ingrediente 59446791</t>
+          <t>Ingrediente 9551f65b</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -797,7 +797,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Producto 27078bf6</t>
+          <t>Producto 1aacee13</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Receta 7dab5b64</t>
+          <t>Receta 0e8c932f</t>
         </is>
       </c>
     </row>
@@ -999,14 +999,14 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46288.29523119341</v>
+        <v>46288.86658869901</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Producto 27078bf6</t>
+          <t>Producto 1aacee13</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1023,14 +1023,14 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46288.62856452673</v>
+        <v>46289.19992203234</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Producto 27078bf6</t>
+          <t>Producto 1aacee13</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1047,14 +1047,14 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46288.96189786007</v>
+        <v>46289.53325536567</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Producto 27078bf6</t>
+          <t>Producto 1aacee13</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1071,14 +1071,14 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46289.29523119341</v>
+        <v>46289.86658869901</v>
       </c>
       <c r="C5" t="n">
         <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Producto 27078bf6</t>
+          <t>Producto 1aacee13</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1095,14 +1095,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46289.62856452673</v>
+        <v>46290.19992203234</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Producto 27078bf6</t>
+          <t>Producto 1aacee13</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1119,14 +1119,14 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46289.96189786007</v>
+        <v>46290.53325536567</v>
       </c>
       <c r="C7" t="n">
         <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Producto 27078bf6</t>
+          <t>Producto 1aacee13</t>
         </is>
       </c>
       <c r="E7" t="n">

</xml_diff>

<commit_message>
All-phase rollout: KDS kanban (Pendientes/En preparación/Listos + status pills), produccion sufficiency matrix (delta + Justo/Suficiente badges + reponer link), clientes tier via SSOT (Bronce), wishlist i18n + sheet-leak removal, ventas-historial kpi_strip + Gs. double-prefix fix, reorder JSON-link removal + plural, bank endpoint-leak removal, KDS heading Spanish
</commit_message>
<xml_diff>
--- a/docs/user-guide/screenshots/all-pages/export-excel.xlsx
+++ b/docs/user-guide/screenshots/all-pages/export-excel.xlsx
@@ -477,7 +477,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ingrediente 9551f65b</t>
+          <t>Ingrediente 37f13e51</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Receta 0e8c932f</t>
+          <t>Receta d6c29c89</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -682,7 +682,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Receta 0e8c932f</t>
+          <t>Receta d6c29c89</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Ingrediente 9551f65b</t>
+          <t>Ingrediente 37f13e51</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -797,7 +797,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Producto 1aacee13</t>
+          <t>Producto 5f9b1800</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Receta 0e8c932f</t>
+          <t>Receta d6c29c89</t>
         </is>
       </c>
     </row>
@@ -999,14 +999,14 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46288.86658869901</v>
+        <v>46288.99773483026</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Producto 1aacee13</t>
+          <t>Producto 5f9b1800</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1023,14 +1023,14 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46289.19992203234</v>
+        <v>46289.3310681636</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Producto 1aacee13</t>
+          <t>Producto 5f9b1800</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1047,14 +1047,14 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46289.53325536567</v>
+        <v>46289.66440149694</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Producto 1aacee13</t>
+          <t>Producto 5f9b1800</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1071,14 +1071,14 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46289.86658869901</v>
+        <v>46289.99773483026</v>
       </c>
       <c r="C5" t="n">
         <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Producto 1aacee13</t>
+          <t>Producto 5f9b1800</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1095,14 +1095,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46290.19992203234</v>
+        <v>46290.3310681636</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Producto 1aacee13</t>
+          <t>Producto 5f9b1800</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1119,14 +1119,14 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46290.53325536567</v>
+        <v>46290.66440149694</v>
       </c>
       <c r="C7" t="n">
         <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Producto 1aacee13</t>
+          <t>Producto 5f9b1800</t>
         </is>
       </c>
       <c r="E7" t="n">

</xml_diff>

<commit_message>
inventario redesign per audit doc: sticky-header contained table (70vh), condensed first column (allergens compact, subcategory/role/dietary/storage → Más info disclosure), Ver/Ajustar/Editar distinct icons
</commit_message>
<xml_diff>
--- a/docs/user-guide/screenshots/all-pages/export-excel.xlsx
+++ b/docs/user-guide/screenshots/all-pages/export-excel.xlsx
@@ -477,7 +477,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ingrediente 37f13e51</t>
+          <t>Ingrediente 840b0455</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Receta d6c29c89</t>
+          <t>Receta 33e39a87</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -682,7 +682,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Receta d6c29c89</t>
+          <t>Receta 33e39a87</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Ingrediente 37f13e51</t>
+          <t>Ingrediente 840b0455</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -797,7 +797,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Producto 5f9b1800</t>
+          <t>Producto 0faba1b0</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Receta d6c29c89</t>
+          <t>Receta 33e39a87</t>
         </is>
       </c>
     </row>
@@ -999,14 +999,14 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>46288.99773483026</v>
+        <v>46289.29964811084</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Producto 5f9b1800</t>
+          <t>Producto 0faba1b0</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1023,14 +1023,14 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46289.3310681636</v>
+        <v>46289.63298144418</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Producto 5f9b1800</t>
+          <t>Producto 0faba1b0</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1047,14 +1047,14 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46289.66440149694</v>
+        <v>46289.96631477751</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Producto 5f9b1800</t>
+          <t>Producto 0faba1b0</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1071,14 +1071,14 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46289.99773483026</v>
+        <v>46290.29964811084</v>
       </c>
       <c r="C5" t="n">
         <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Producto 5f9b1800</t>
+          <t>Producto 0faba1b0</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1095,14 +1095,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46290.3310681636</v>
+        <v>46290.63298144418</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Producto 5f9b1800</t>
+          <t>Producto 0faba1b0</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1119,14 +1119,14 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46290.66440149694</v>
+        <v>46290.96631477751</v>
       </c>
       <c r="C7" t="n">
         <v>1</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Producto 5f9b1800</t>
+          <t>Producto 0faba1b0</t>
         </is>
       </c>
       <c r="E7" t="n">

</xml_diff>